<commit_message>
fix(bosmax_command_centre_repository_governance): mirror part2 lipsync retained pack [Mandor-Gate: PASSED | Sandbox: Manual]
</commit_message>
<xml_diff>
--- a/Bosmax-Command-Centre/knowledge-pack/copywriting/COPYWRITING_MASTER_BOSMAX.xlsx
+++ b/Bosmax-Command-Centre/knowledge-pack/copywriting/COPYWRITING_MASTER_BOSMAX.xlsx
@@ -12,6 +12,7 @@
     <sheet name="RISK_VALIDATION" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="SOURCE_MAP" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="QA_REPORT" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="ContinuationSafeCopy" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -24,7 +25,7 @@
     <numFmt numFmtId="164" formatCode="_-&quot;RM&quot;* #,##0.00_-;\-&quot;RM&quot;* #,##0.00_-;_-&quot;RM&quot;* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="165" formatCode="_-&quot;RM&quot;* #,##0_-;\-&quot;RM&quot;* #,##0_-;_-&quot;RM&quot;* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="23">
     <font>
       <name val="Calibri"/>
       <charset val="134"/>
@@ -187,6 +188,9 @@
       <name val="Calibri"/>
       <b val="1"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="33">
@@ -637,9 +641,10 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -10662,4 +10667,103 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>part2_dialogue_6s_malay</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>part2_dialogue_8s_malay</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>part2_word_count</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>part2_lipsync_safe_flag</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>part2_cta_short</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>part2_no_vo_flag</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>part2_notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Kecil je macam lip balm, senang standby. Tap tengok harga sekarang, boss.</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D2" t="b">
+        <v>1</v>
+      </c>
+      <c r="E2" t="b">
+        <v>1</v>
+      </c>
+      <c r="F2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>BOSMAX Serum Part 2 closes the existing practical carry cue only; no new metaphor or new proof.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Kecil je macam lip balm, senang bawa dan terus nampak kemas. Tap tengok harga sekarang, boss.</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>16</v>
+      </c>
+      <c r="D3" t="b">
+        <v>1</v>
+      </c>
+      <c r="E3" t="b">
+        <v>1</v>
+      </c>
+      <c r="F3" t="b">
+        <v>1</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Google Flow 8s continuation keeps the on-camera carry cue and a short direct CTA.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>